<commit_message>
update: 周三 2026/06/03 10:45:08.75
</commit_message>
<xml_diff>
--- a/source/4、后勤及职能占比/后勤及职能占比-5月.xlsx
+++ b/source/4、后勤及职能占比/后勤及职能占比-5月.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4551" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4854" uniqueCount="97">
   <si>
     <t>数据日期</t>
   </si>
@@ -313,6 +313,12 @@
   </si>
   <si>
     <t>2026-05-29</t>
+  </si>
+  <si>
+    <t>2026-05-30</t>
+  </si>
+  <si>
+    <t>2026-05-31</t>
   </si>
 </sst>
 </file>
@@ -1246,7 +1252,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:F1516"/>
+  <dimension ref="A1:F1617"/>
   <sheetFormatPr defaultColWidth="12.6363636363636" defaultRowHeight="20" customHeight="1" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="16384" width="12.6363636363636" style="1" customWidth="1"/>
@@ -31569,6 +31575,2026 @@
         <v>92</v>
       </c>
       <c r="F1516" s="1">
+        <v>8.2</v>
+      </c>
+    </row>
+    <row r="1517" customHeight="1" spans="1:6">
+      <c r="A1517" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1517" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1517" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1517" s="1">
+        <v>299</v>
+      </c>
+      <c r="E1517" s="1">
+        <v>72</v>
+      </c>
+      <c r="F1517" s="1">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="1518" customHeight="1" spans="1:6">
+      <c r="A1518" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1518" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1518" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1518" s="1">
+        <v>333</v>
+      </c>
+      <c r="E1518" s="1">
+        <v>53</v>
+      </c>
+      <c r="F1518" s="1">
+        <v>15.9</v>
+      </c>
+    </row>
+    <row r="1519" customHeight="1" spans="1:6">
+      <c r="A1519" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1519" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C1519" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1519" s="1">
+        <v>359</v>
+      </c>
+      <c r="E1519" s="1">
+        <v>52</v>
+      </c>
+      <c r="F1519" s="1">
+        <v>14.4</v>
+      </c>
+    </row>
+    <row r="1520" customHeight="1" spans="1:6">
+      <c r="A1520" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1520" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1520" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1520" s="1">
+        <v>441</v>
+      </c>
+      <c r="E1520" s="1">
+        <v>63</v>
+      </c>
+      <c r="F1520" s="1">
+        <v>14.2</v>
+      </c>
+    </row>
+    <row r="1521" customHeight="1" spans="1:6">
+      <c r="A1521" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1521" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1521" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1521" s="1">
+        <v>353</v>
+      </c>
+      <c r="E1521" s="1">
+        <v>50</v>
+      </c>
+      <c r="F1521" s="1">
+        <v>14.1</v>
+      </c>
+    </row>
+    <row r="1522" customHeight="1" spans="1:6">
+      <c r="A1522" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1522" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1522" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1522" s="1">
+        <v>493</v>
+      </c>
+      <c r="E1522" s="1">
+        <v>70</v>
+      </c>
+      <c r="F1522" s="1">
+        <v>14.1</v>
+      </c>
+    </row>
+    <row r="1523" customHeight="1" spans="1:6">
+      <c r="A1523" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1523" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1523" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1523" s="1">
+        <v>423</v>
+      </c>
+      <c r="E1523" s="1">
+        <v>59</v>
+      </c>
+      <c r="F1523" s="1">
+        <v>13.9</v>
+      </c>
+    </row>
+    <row r="1524" customHeight="1" spans="1:6">
+      <c r="A1524" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1524" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1524" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1524" s="1">
+        <v>315</v>
+      </c>
+      <c r="E1524" s="1">
+        <v>44</v>
+      </c>
+      <c r="F1524" s="1">
+        <v>13.9</v>
+      </c>
+    </row>
+    <row r="1525" customHeight="1" spans="1:6">
+      <c r="A1525" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1525" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1525" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1525" s="1">
+        <v>246</v>
+      </c>
+      <c r="E1525" s="1">
+        <v>34</v>
+      </c>
+      <c r="F1525" s="1">
+        <v>13.8</v>
+      </c>
+    </row>
+    <row r="1526" customHeight="1" spans="1:6">
+      <c r="A1526" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1526" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1526" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1526" s="1">
+        <v>405</v>
+      </c>
+      <c r="E1526" s="1">
+        <v>56</v>
+      </c>
+      <c r="F1526" s="1">
+        <v>13.8</v>
+      </c>
+    </row>
+    <row r="1527" customHeight="1" spans="1:6">
+      <c r="A1527" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1527" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1527" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1527" s="1">
+        <v>586</v>
+      </c>
+      <c r="E1527" s="1">
+        <v>80</v>
+      </c>
+      <c r="F1527" s="1">
+        <v>13.6</v>
+      </c>
+    </row>
+    <row r="1528" customHeight="1" spans="1:6">
+      <c r="A1528" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1528" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1528" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1528" s="1">
+        <v>173</v>
+      </c>
+      <c r="E1528" s="1">
+        <v>23</v>
+      </c>
+      <c r="F1528" s="1">
+        <v>13.2</v>
+      </c>
+    </row>
+    <row r="1529" customHeight="1" spans="1:6">
+      <c r="A1529" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1529" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1529" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1529" s="1">
+        <v>478</v>
+      </c>
+      <c r="E1529" s="1">
+        <v>63</v>
+      </c>
+      <c r="F1529" s="1">
+        <v>13.1</v>
+      </c>
+    </row>
+    <row r="1530" customHeight="1" spans="1:6">
+      <c r="A1530" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1530" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1530" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1530" s="1">
+        <v>396</v>
+      </c>
+      <c r="E1530" s="1">
+        <v>52</v>
+      </c>
+      <c r="F1530" s="1">
+        <v>13.1</v>
+      </c>
+    </row>
+    <row r="1531" customHeight="1" spans="1:6">
+      <c r="A1531" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1531" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1531" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1531" s="1">
+        <v>451</v>
+      </c>
+      <c r="E1531" s="1">
+        <v>59</v>
+      </c>
+      <c r="F1531" s="1">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="1532" customHeight="1" spans="1:6">
+      <c r="A1532" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1532" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C1532" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1532" s="1">
+        <v>381</v>
+      </c>
+      <c r="E1532" s="1">
+        <v>48</v>
+      </c>
+      <c r="F1532" s="1">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="1533" customHeight="1" spans="1:6">
+      <c r="A1533" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1533" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1533" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1533" s="1">
+        <v>408</v>
+      </c>
+      <c r="E1533" s="1">
+        <v>51</v>
+      </c>
+      <c r="F1533" s="1">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="1534" customHeight="1" spans="1:6">
+      <c r="A1534" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1534" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C1534" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1534" s="1">
+        <v>456</v>
+      </c>
+      <c r="E1534" s="1">
+        <v>57</v>
+      </c>
+      <c r="F1534" s="1">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="1535" customHeight="1" spans="1:6">
+      <c r="A1535" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1535" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C1535" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1535" s="1">
+        <v>610</v>
+      </c>
+      <c r="E1535" s="1">
+        <v>76</v>
+      </c>
+      <c r="F1535" s="1">
+        <v>12.4</v>
+      </c>
+    </row>
+    <row r="1536" customHeight="1" spans="1:6">
+      <c r="A1536" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1536" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C1536" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1536" s="1">
+        <v>315</v>
+      </c>
+      <c r="E1536" s="1">
+        <v>39</v>
+      </c>
+      <c r="F1536" s="1">
+        <v>12.3</v>
+      </c>
+    </row>
+    <row r="1537" customHeight="1" spans="1:6">
+      <c r="A1537" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1537" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C1537" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1537" s="1">
+        <v>638</v>
+      </c>
+      <c r="E1537" s="1">
+        <v>79</v>
+      </c>
+      <c r="F1537" s="1">
+        <v>12.3</v>
+      </c>
+    </row>
+    <row r="1538" customHeight="1" spans="1:6">
+      <c r="A1538" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1538" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1538" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1538" s="1">
+        <v>842</v>
+      </c>
+      <c r="E1538" s="1">
+        <v>103</v>
+      </c>
+      <c r="F1538" s="1">
+        <v>12.2</v>
+      </c>
+    </row>
+    <row r="1539" customHeight="1" spans="1:6">
+      <c r="A1539" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1539" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C1539" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1539" s="1">
+        <v>758</v>
+      </c>
+      <c r="E1539" s="1">
+        <v>92</v>
+      </c>
+      <c r="F1539" s="1">
+        <v>12.1</v>
+      </c>
+    </row>
+    <row r="1540" customHeight="1" spans="1:6">
+      <c r="A1540" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1540" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C1540" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1540" s="1">
+        <v>790</v>
+      </c>
+      <c r="E1540" s="1">
+        <v>95</v>
+      </c>
+      <c r="F1540" s="1">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1541" customHeight="1" spans="1:6">
+      <c r="A1541" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1541" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1541" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1541" s="1">
+        <v>1137</v>
+      </c>
+      <c r="E1541" s="1">
+        <v>131</v>
+      </c>
+      <c r="F1541" s="1">
+        <v>11.5</v>
+      </c>
+    </row>
+    <row r="1542" customHeight="1" spans="1:6">
+      <c r="A1542" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1542" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C1542" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1542" s="1">
+        <v>1352</v>
+      </c>
+      <c r="E1542" s="1">
+        <v>155</v>
+      </c>
+      <c r="F1542" s="1">
+        <v>11.4</v>
+      </c>
+    </row>
+    <row r="1543" customHeight="1" spans="1:6">
+      <c r="A1543" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1543" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1543" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1543" s="1">
+        <v>585</v>
+      </c>
+      <c r="E1543" s="1">
+        <v>66</v>
+      </c>
+      <c r="F1543" s="1">
+        <v>11.2</v>
+      </c>
+    </row>
+    <row r="1544" customHeight="1" spans="1:6">
+      <c r="A1544" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1544" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1544" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1544" s="1">
+        <v>957</v>
+      </c>
+      <c r="E1544" s="1">
+        <v>105</v>
+      </c>
+      <c r="F1544" s="1">
+        <v>10.9</v>
+      </c>
+    </row>
+    <row r="1545" customHeight="1" spans="1:6">
+      <c r="A1545" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1545" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C1545" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1545" s="1">
+        <v>440</v>
+      </c>
+      <c r="E1545" s="1">
+        <v>47</v>
+      </c>
+      <c r="F1545" s="1">
+        <v>10.6</v>
+      </c>
+    </row>
+    <row r="1546" customHeight="1" spans="1:6">
+      <c r="A1546" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1546" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C1546" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1546" s="1">
+        <v>531</v>
+      </c>
+      <c r="E1546" s="1">
+        <v>56</v>
+      </c>
+      <c r="F1546" s="1">
+        <v>10.5</v>
+      </c>
+    </row>
+    <row r="1547" customHeight="1" spans="1:6">
+      <c r="A1547" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1547" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C1547" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1547" s="1">
+        <v>613</v>
+      </c>
+      <c r="E1547" s="1">
+        <v>64</v>
+      </c>
+      <c r="F1547" s="1">
+        <v>10.4</v>
+      </c>
+    </row>
+    <row r="1548" customHeight="1" spans="1:6">
+      <c r="A1548" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1548" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1548" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1548" s="1">
+        <v>716</v>
+      </c>
+      <c r="E1548" s="1">
+        <v>75</v>
+      </c>
+      <c r="F1548" s="1">
+        <v>10.4</v>
+      </c>
+    </row>
+    <row r="1549" customHeight="1" spans="1:6">
+      <c r="A1549" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1549" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C1549" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1549" s="1">
+        <v>967</v>
+      </c>
+      <c r="E1549" s="1">
+        <v>100</v>
+      </c>
+      <c r="F1549" s="1">
+        <v>10.3</v>
+      </c>
+    </row>
+    <row r="1550" customHeight="1" spans="1:6">
+      <c r="A1550" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1550" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C1550" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1550" s="1">
+        <v>599</v>
+      </c>
+      <c r="E1550" s="1">
+        <v>62</v>
+      </c>
+      <c r="F1550" s="1">
+        <v>10.3</v>
+      </c>
+    </row>
+    <row r="1551" customHeight="1" spans="1:6">
+      <c r="A1551" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1551" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C1551" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1551" s="1">
+        <v>615</v>
+      </c>
+      <c r="E1551" s="1">
+        <v>63</v>
+      </c>
+      <c r="F1551" s="1">
+        <v>10.2</v>
+      </c>
+    </row>
+    <row r="1552" customHeight="1" spans="1:6">
+      <c r="A1552" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1552" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C1552" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1552" s="1">
+        <v>1054</v>
+      </c>
+      <c r="E1552" s="1">
+        <v>108</v>
+      </c>
+      <c r="F1552" s="1">
+        <v>10.2</v>
+      </c>
+    </row>
+    <row r="1553" customHeight="1" spans="1:6">
+      <c r="A1553" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1553" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C1553" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1553" s="1">
+        <v>1047</v>
+      </c>
+      <c r="E1553" s="1">
+        <v>106</v>
+      </c>
+      <c r="F1553" s="1">
+        <v>10.1</v>
+      </c>
+    </row>
+    <row r="1554" customHeight="1" spans="1:6">
+      <c r="A1554" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1554" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C1554" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1554" s="1">
+        <v>1257</v>
+      </c>
+      <c r="E1554" s="1">
+        <v>124</v>
+      </c>
+      <c r="F1554" s="1">
+        <v>9.8</v>
+      </c>
+    </row>
+    <row r="1555" customHeight="1" spans="1:6">
+      <c r="A1555" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1555" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C1555" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1555" s="1">
+        <v>1196</v>
+      </c>
+      <c r="E1555" s="1">
+        <v>118</v>
+      </c>
+      <c r="F1555" s="1">
+        <v>9.8</v>
+      </c>
+    </row>
+    <row r="1556" customHeight="1" spans="1:6">
+      <c r="A1556" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1556" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C1556" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1556" s="1">
+        <v>1051</v>
+      </c>
+      <c r="E1556" s="1">
+        <v>100</v>
+      </c>
+      <c r="F1556" s="1">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="1557" customHeight="1" spans="1:6">
+      <c r="A1557" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1557" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C1557" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1557" s="1">
+        <v>1675</v>
+      </c>
+      <c r="E1557" s="1">
+        <v>160</v>
+      </c>
+      <c r="F1557" s="1">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="1558" customHeight="1" spans="1:6">
+      <c r="A1558" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1558" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C1558" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1558" s="1">
+        <v>1284</v>
+      </c>
+      <c r="E1558" s="1">
+        <v>121</v>
+      </c>
+      <c r="F1558" s="1">
+        <v>9.4</v>
+      </c>
+    </row>
+    <row r="1559" customHeight="1" spans="1:6">
+      <c r="A1559" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1559" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C1559" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1559" s="1">
+        <v>892</v>
+      </c>
+      <c r="E1559" s="1">
+        <v>83</v>
+      </c>
+      <c r="F1559" s="1">
+        <v>9.3</v>
+      </c>
+    </row>
+    <row r="1560" customHeight="1" spans="1:6">
+      <c r="A1560" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1560" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C1560" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1560" s="1">
+        <v>1544</v>
+      </c>
+      <c r="E1560" s="1">
+        <v>144</v>
+      </c>
+      <c r="F1560" s="1">
+        <v>9.3</v>
+      </c>
+    </row>
+    <row r="1561" customHeight="1" spans="1:6">
+      <c r="A1561" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1561" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C1561" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1561" s="1">
+        <v>1177</v>
+      </c>
+      <c r="E1561" s="1">
+        <v>108</v>
+      </c>
+      <c r="F1561" s="1">
+        <v>9.1</v>
+      </c>
+    </row>
+    <row r="1562" customHeight="1" spans="1:6">
+      <c r="A1562" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1562" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C1562" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1562" s="1">
+        <v>1866</v>
+      </c>
+      <c r="E1562" s="1">
+        <v>168</v>
+      </c>
+      <c r="F1562" s="1">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1563" customHeight="1" spans="1:6">
+      <c r="A1563" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1563" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C1563" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1563" s="1">
+        <v>1272</v>
+      </c>
+      <c r="E1563" s="1">
+        <v>111</v>
+      </c>
+      <c r="F1563" s="1">
+        <v>8.7</v>
+      </c>
+    </row>
+    <row r="1564" customHeight="1" spans="1:6">
+      <c r="A1564" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1564" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C1564" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1564" s="1">
+        <v>1540</v>
+      </c>
+      <c r="E1564" s="1">
+        <v>133</v>
+      </c>
+      <c r="F1564" s="1">
+        <v>8.6</v>
+      </c>
+    </row>
+    <row r="1565" customHeight="1" spans="1:6">
+      <c r="A1565" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1565" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C1565" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1565" s="1">
+        <v>1041</v>
+      </c>
+      <c r="E1565" s="1">
+        <v>90</v>
+      </c>
+      <c r="F1565" s="1">
+        <v>8.6</v>
+      </c>
+    </row>
+    <row r="1566" customHeight="1" spans="1:6">
+      <c r="A1566" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1566" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1566" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1566" s="1">
+        <v>959</v>
+      </c>
+      <c r="E1566" s="1">
+        <v>82</v>
+      </c>
+      <c r="F1566" s="1">
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="1567" customHeight="1" spans="1:6">
+      <c r="A1567" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1567" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C1567" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1567" s="1">
+        <v>1109</v>
+      </c>
+      <c r="E1567" s="1">
+        <v>92</v>
+      </c>
+      <c r="F1567" s="1">
+        <v>8.2</v>
+      </c>
+    </row>
+    <row r="1568" customHeight="1" spans="1:6">
+      <c r="A1568" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1568" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1568" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1568" s="1">
+        <v>301</v>
+      </c>
+      <c r="E1568" s="1">
+        <v>72</v>
+      </c>
+      <c r="F1568" s="1">
+        <v>23.9</v>
+      </c>
+    </row>
+    <row r="1569" customHeight="1" spans="1:6">
+      <c r="A1569" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1569" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1569" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1569" s="1">
+        <v>333</v>
+      </c>
+      <c r="E1569" s="1">
+        <v>53</v>
+      </c>
+      <c r="F1569" s="1">
+        <v>15.9</v>
+      </c>
+    </row>
+    <row r="1570" customHeight="1" spans="1:6">
+      <c r="A1570" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1570" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C1570" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1570" s="1">
+        <v>359</v>
+      </c>
+      <c r="E1570" s="1">
+        <v>52</v>
+      </c>
+      <c r="F1570" s="1">
+        <v>14.4</v>
+      </c>
+    </row>
+    <row r="1571" customHeight="1" spans="1:6">
+      <c r="A1571" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1571" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1571" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1571" s="1">
+        <v>435</v>
+      </c>
+      <c r="E1571" s="1">
+        <v>63</v>
+      </c>
+      <c r="F1571" s="1">
+        <v>14.4</v>
+      </c>
+    </row>
+    <row r="1572" customHeight="1" spans="1:6">
+      <c r="A1572" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1572" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1572" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1572" s="1">
+        <v>492</v>
+      </c>
+      <c r="E1572" s="1">
+        <v>70</v>
+      </c>
+      <c r="F1572" s="1">
+        <v>14.2</v>
+      </c>
+    </row>
+    <row r="1573" customHeight="1" spans="1:6">
+      <c r="A1573" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1573" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1573" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1573" s="1">
+        <v>354</v>
+      </c>
+      <c r="E1573" s="1">
+        <v>50</v>
+      </c>
+      <c r="F1573" s="1">
+        <v>14.1</v>
+      </c>
+    </row>
+    <row r="1574" customHeight="1" spans="1:6">
+      <c r="A1574" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1574" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1574" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1574" s="1">
+        <v>314</v>
+      </c>
+      <c r="E1574" s="1">
+        <v>44</v>
+      </c>
+      <c r="F1574" s="1">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="1575" customHeight="1" spans="1:6">
+      <c r="A1575" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1575" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1575" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1575" s="1">
+        <v>245</v>
+      </c>
+      <c r="E1575" s="1">
+        <v>34</v>
+      </c>
+      <c r="F1575" s="1">
+        <v>13.8</v>
+      </c>
+    </row>
+    <row r="1576" customHeight="1" spans="1:6">
+      <c r="A1576" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1576" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1576" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1576" s="1">
+        <v>425</v>
+      </c>
+      <c r="E1576" s="1">
+        <v>59</v>
+      </c>
+      <c r="F1576" s="1">
+        <v>13.8</v>
+      </c>
+    </row>
+    <row r="1577" customHeight="1" spans="1:6">
+      <c r="A1577" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1577" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1577" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1577" s="1">
+        <v>405</v>
+      </c>
+      <c r="E1577" s="1">
+        <v>56</v>
+      </c>
+      <c r="F1577" s="1">
+        <v>13.8</v>
+      </c>
+    </row>
+    <row r="1578" customHeight="1" spans="1:6">
+      <c r="A1578" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1578" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1578" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1578" s="1">
+        <v>586</v>
+      </c>
+      <c r="E1578" s="1">
+        <v>80</v>
+      </c>
+      <c r="F1578" s="1">
+        <v>13.6</v>
+      </c>
+    </row>
+    <row r="1579" customHeight="1" spans="1:6">
+      <c r="A1579" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1579" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1579" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1579" s="1">
+        <v>173</v>
+      </c>
+      <c r="E1579" s="1">
+        <v>23</v>
+      </c>
+      <c r="F1579" s="1">
+        <v>13.2</v>
+      </c>
+    </row>
+    <row r="1580" customHeight="1" spans="1:6">
+      <c r="A1580" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1580" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1580" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1580" s="1">
+        <v>478</v>
+      </c>
+      <c r="E1580" s="1">
+        <v>63</v>
+      </c>
+      <c r="F1580" s="1">
+        <v>13.1</v>
+      </c>
+    </row>
+    <row r="1581" customHeight="1" spans="1:6">
+      <c r="A1581" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1581" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1581" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1581" s="1">
+        <v>396</v>
+      </c>
+      <c r="E1581" s="1">
+        <v>52</v>
+      </c>
+      <c r="F1581" s="1">
+        <v>13.1</v>
+      </c>
+    </row>
+    <row r="1582" customHeight="1" spans="1:6">
+      <c r="A1582" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1582" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1582" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1582" s="1">
+        <v>452</v>
+      </c>
+      <c r="E1582" s="1">
+        <v>59</v>
+      </c>
+      <c r="F1582" s="1">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="1583" customHeight="1" spans="1:6">
+      <c r="A1583" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1583" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C1583" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1583" s="1">
+        <v>381</v>
+      </c>
+      <c r="E1583" s="1">
+        <v>48</v>
+      </c>
+      <c r="F1583" s="1">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="1584" customHeight="1" spans="1:6">
+      <c r="A1584" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1584" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1584" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1584" s="1">
+        <v>406</v>
+      </c>
+      <c r="E1584" s="1">
+        <v>51</v>
+      </c>
+      <c r="F1584" s="1">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="1585" customHeight="1" spans="1:6">
+      <c r="A1585" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1585" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C1585" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1585" s="1">
+        <v>456</v>
+      </c>
+      <c r="E1585" s="1">
+        <v>57</v>
+      </c>
+      <c r="F1585" s="1">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="1586" customHeight="1" spans="1:6">
+      <c r="A1586" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1586" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C1586" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1586" s="1">
+        <v>605</v>
+      </c>
+      <c r="E1586" s="1">
+        <v>76</v>
+      </c>
+      <c r="F1586" s="1">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="1587" customHeight="1" spans="1:6">
+      <c r="A1587" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1587" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C1587" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1587" s="1">
+        <v>315</v>
+      </c>
+      <c r="E1587" s="1">
+        <v>39</v>
+      </c>
+      <c r="F1587" s="1">
+        <v>12.3</v>
+      </c>
+    </row>
+    <row r="1588" customHeight="1" spans="1:6">
+      <c r="A1588" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1588" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C1588" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1588" s="1">
+        <v>638</v>
+      </c>
+      <c r="E1588" s="1">
+        <v>79</v>
+      </c>
+      <c r="F1588" s="1">
+        <v>12.3</v>
+      </c>
+    </row>
+    <row r="1589" customHeight="1" spans="1:6">
+      <c r="A1589" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1589" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1589" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1589" s="1">
+        <v>842</v>
+      </c>
+      <c r="E1589" s="1">
+        <v>103</v>
+      </c>
+      <c r="F1589" s="1">
+        <v>12.2</v>
+      </c>
+    </row>
+    <row r="1590" customHeight="1" spans="1:6">
+      <c r="A1590" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1590" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C1590" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1590" s="1">
+        <v>758</v>
+      </c>
+      <c r="E1590" s="1">
+        <v>92</v>
+      </c>
+      <c r="F1590" s="1">
+        <v>12.1</v>
+      </c>
+    </row>
+    <row r="1591" customHeight="1" spans="1:6">
+      <c r="A1591" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1591" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C1591" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1591" s="1">
+        <v>790</v>
+      </c>
+      <c r="E1591" s="1">
+        <v>95</v>
+      </c>
+      <c r="F1591" s="1">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1592" customHeight="1" spans="1:6">
+      <c r="A1592" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1592" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1592" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1592" s="1">
+        <v>1138</v>
+      </c>
+      <c r="E1592" s="1">
+        <v>131</v>
+      </c>
+      <c r="F1592" s="1">
+        <v>11.5</v>
+      </c>
+    </row>
+    <row r="1593" customHeight="1" spans="1:6">
+      <c r="A1593" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1593" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C1593" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1593" s="1">
+        <v>1351</v>
+      </c>
+      <c r="E1593" s="1">
+        <v>154</v>
+      </c>
+      <c r="F1593" s="1">
+        <v>11.3</v>
+      </c>
+    </row>
+    <row r="1594" customHeight="1" spans="1:6">
+      <c r="A1594" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1594" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1594" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1594" s="1">
+        <v>585</v>
+      </c>
+      <c r="E1594" s="1">
+        <v>66</v>
+      </c>
+      <c r="F1594" s="1">
+        <v>11.2</v>
+      </c>
+    </row>
+    <row r="1595" customHeight="1" spans="1:6">
+      <c r="A1595" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1595" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1595" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1595" s="1">
+        <v>957</v>
+      </c>
+      <c r="E1595" s="1">
+        <v>105</v>
+      </c>
+      <c r="F1595" s="1">
+        <v>10.9</v>
+      </c>
+    </row>
+    <row r="1596" customHeight="1" spans="1:6">
+      <c r="A1596" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1596" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C1596" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1596" s="1">
+        <v>439</v>
+      </c>
+      <c r="E1596" s="1">
+        <v>47</v>
+      </c>
+      <c r="F1596" s="1">
+        <v>10.7</v>
+      </c>
+    </row>
+    <row r="1597" customHeight="1" spans="1:6">
+      <c r="A1597" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1597" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C1597" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1597" s="1">
+        <v>533</v>
+      </c>
+      <c r="E1597" s="1">
+        <v>56</v>
+      </c>
+      <c r="F1597" s="1">
+        <v>10.5</v>
+      </c>
+    </row>
+    <row r="1598" customHeight="1" spans="1:6">
+      <c r="A1598" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1598" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C1598" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1598" s="1">
+        <v>612</v>
+      </c>
+      <c r="E1598" s="1">
+        <v>64</v>
+      </c>
+      <c r="F1598" s="1">
+        <v>10.4</v>
+      </c>
+    </row>
+    <row r="1599" customHeight="1" spans="1:6">
+      <c r="A1599" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1599" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C1599" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1599" s="1">
+        <v>599</v>
+      </c>
+      <c r="E1599" s="1">
+        <v>62</v>
+      </c>
+      <c r="F1599" s="1">
+        <v>10.3</v>
+      </c>
+    </row>
+    <row r="1600" customHeight="1" spans="1:6">
+      <c r="A1600" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1600" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C1600" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1600" s="1">
+        <v>966</v>
+      </c>
+      <c r="E1600" s="1">
+        <v>100</v>
+      </c>
+      <c r="F1600" s="1">
+        <v>10.3</v>
+      </c>
+    </row>
+    <row r="1601" customHeight="1" spans="1:6">
+      <c r="A1601" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1601" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C1601" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1601" s="1">
+        <v>1054</v>
+      </c>
+      <c r="E1601" s="1">
+        <v>108</v>
+      </c>
+      <c r="F1601" s="1">
+        <v>10.2</v>
+      </c>
+    </row>
+    <row r="1602" customHeight="1" spans="1:6">
+      <c r="A1602" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1602" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C1602" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1602" s="1">
+        <v>614</v>
+      </c>
+      <c r="E1602" s="1">
+        <v>63</v>
+      </c>
+      <c r="F1602" s="1">
+        <v>10.2</v>
+      </c>
+    </row>
+    <row r="1603" customHeight="1" spans="1:6">
+      <c r="A1603" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1603" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C1603" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1603" s="1">
+        <v>1049</v>
+      </c>
+      <c r="E1603" s="1">
+        <v>106</v>
+      </c>
+      <c r="F1603" s="1">
+        <v>10.1</v>
+      </c>
+    </row>
+    <row r="1604" customHeight="1" spans="1:6">
+      <c r="A1604" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1604" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C1604" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1604" s="1">
+        <v>1260</v>
+      </c>
+      <c r="E1604" s="1">
+        <v>124</v>
+      </c>
+      <c r="F1604" s="1">
+        <v>9.8</v>
+      </c>
+    </row>
+    <row r="1605" customHeight="1" spans="1:6">
+      <c r="A1605" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1605" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C1605" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1605" s="1">
+        <v>1196</v>
+      </c>
+      <c r="E1605" s="1">
+        <v>118</v>
+      </c>
+      <c r="F1605" s="1">
+        <v>9.8</v>
+      </c>
+    </row>
+    <row r="1606" customHeight="1" spans="1:6">
+      <c r="A1606" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1606" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C1606" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1606" s="1">
+        <v>1051</v>
+      </c>
+      <c r="E1606" s="1">
+        <v>100</v>
+      </c>
+      <c r="F1606" s="1">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="1607" customHeight="1" spans="1:6">
+      <c r="A1607" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1607" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C1607" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1607" s="1">
+        <v>1674</v>
+      </c>
+      <c r="E1607" s="1">
+        <v>160</v>
+      </c>
+      <c r="F1607" s="1">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="1608" customHeight="1" spans="1:6">
+      <c r="A1608" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1608" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C1608" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1608" s="1">
+        <v>1284</v>
+      </c>
+      <c r="E1608" s="1">
+        <v>121</v>
+      </c>
+      <c r="F1608" s="1">
+        <v>9.4</v>
+      </c>
+    </row>
+    <row r="1609" customHeight="1" spans="1:6">
+      <c r="A1609" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1609" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C1609" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1609" s="1">
+        <v>892</v>
+      </c>
+      <c r="E1609" s="1">
+        <v>83</v>
+      </c>
+      <c r="F1609" s="1">
+        <v>9.3</v>
+      </c>
+    </row>
+    <row r="1610" customHeight="1" spans="1:6">
+      <c r="A1610" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1610" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C1610" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1610" s="1">
+        <v>1550</v>
+      </c>
+      <c r="E1610" s="1">
+        <v>145</v>
+      </c>
+      <c r="F1610" s="1">
+        <v>9.3</v>
+      </c>
+    </row>
+    <row r="1611" customHeight="1" spans="1:6">
+      <c r="A1611" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1611" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C1611" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1611" s="1">
+        <v>1866</v>
+      </c>
+      <c r="E1611" s="1">
+        <v>168</v>
+      </c>
+      <c r="F1611" s="1">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1612" customHeight="1" spans="1:6">
+      <c r="A1612" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1612" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C1612" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1612" s="1">
+        <v>1176</v>
+      </c>
+      <c r="E1612" s="1">
+        <v>106</v>
+      </c>
+      <c r="F1612" s="1">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1613" customHeight="1" spans="1:6">
+      <c r="A1613" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1613" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C1613" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1613" s="1">
+        <v>1271</v>
+      </c>
+      <c r="E1613" s="1">
+        <v>111</v>
+      </c>
+      <c r="F1613" s="1">
+        <v>8.7</v>
+      </c>
+    </row>
+    <row r="1614" customHeight="1" spans="1:6">
+      <c r="A1614" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1614" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C1614" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1614" s="1">
+        <v>1540</v>
+      </c>
+      <c r="E1614" s="1">
+        <v>133</v>
+      </c>
+      <c r="F1614" s="1">
+        <v>8.6</v>
+      </c>
+    </row>
+    <row r="1615" customHeight="1" spans="1:6">
+      <c r="A1615" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1615" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C1615" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1615" s="1">
+        <v>1042</v>
+      </c>
+      <c r="E1615" s="1">
+        <v>90</v>
+      </c>
+      <c r="F1615" s="1">
+        <v>8.6</v>
+      </c>
+    </row>
+    <row r="1616" customHeight="1" spans="1:6">
+      <c r="A1616" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1616" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1616" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1616" s="1">
+        <v>962</v>
+      </c>
+      <c r="E1616" s="1">
+        <v>82</v>
+      </c>
+      <c r="F1616" s="1">
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="1617" customHeight="1" spans="1:6">
+      <c r="A1617" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1617" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C1617" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1617" s="1">
+        <v>1109</v>
+      </c>
+      <c r="E1617" s="1">
+        <v>92</v>
+      </c>
+      <c r="F1617" s="1">
         <v>8.2</v>
       </c>
     </row>

</xml_diff>